<commit_message>
#167 TOP and Bottom Board eSpark BOM Updated.
</commit_message>
<xml_diff>
--- a/Design-Files/SM_Bottom_Board_v3.4/BOM/eSpark-BOM-Bottom (20 Board).xlsx
+++ b/Design-Files/SM_Bottom_Board_v3.4/BOM/eSpark-BOM-Bottom (20 Board).xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="226">
   <si>
     <t>Component list</t>
   </si>
@@ -199,9 +199,6 @@
     <t>IC TRANSCEIVER HALF 1/1 8SOIC</t>
   </si>
   <si>
-    <t>SENSOR ANGLE 360DEG SMD</t>
-  </si>
-  <si>
     <t>IMUACCEL/GYROI2C/SPI14LGA</t>
   </si>
   <si>
@@ -337,9 +334,6 @@
     <t>SN65HVDA1040AQDRQ1</t>
   </si>
   <si>
-    <t>TLE5012BE1000</t>
-  </si>
-  <si>
     <t>LSM6DSLTR</t>
   </si>
   <si>
@@ -400,9 +394,6 @@
     <t>Texas Instruments</t>
   </si>
   <si>
-    <t>Infineon</t>
-  </si>
-  <si>
     <t>Microchip</t>
   </si>
   <si>
@@ -583,9 +574,6 @@
     <t>C188675</t>
   </si>
   <si>
-    <t>C123083</t>
-  </si>
-  <si>
     <t>C100024</t>
   </si>
   <si>
@@ -601,9 +589,6 @@
     <t>100 LQFP</t>
   </si>
   <si>
-    <t>QFN-24</t>
-  </si>
-  <si>
     <t>LGA-14</t>
   </si>
   <si>
@@ -712,7 +697,19 @@
     <t>4.7K</t>
   </si>
   <si>
-    <t>C2, C3, C4, C5, C6, C7, C8, C9, C10, C11, C15, C33, C34, C36, C37, C50 , CF1 , C21</t>
+    <t>AEAT-9955</t>
+  </si>
+  <si>
+    <t>C2, C3, C4, C5, C6, C7, C8, C9, C10, C11, C15, C33, C34, C36, C37, C50, C22, CF1, C21</t>
+  </si>
+  <si>
+    <t>18B SINGLE MAG ENC MULTIPLE AXIS</t>
+  </si>
+  <si>
+    <t>32-QFN (5x5)</t>
+  </si>
+  <si>
+    <t>Broadcom Limited</t>
   </si>
 </sst>
 </file>
@@ -933,7 +930,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="24">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -1189,25 +1186,12 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1309,10 +1293,6 @@
     <xf numFmtId="165" fontId="18" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -1419,6 +1399,24 @@
     <xf numFmtId="0" fontId="24" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1445,27 +1443,7 @@
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="22" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1808,7 +1786,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:V43"/>
+  <dimension ref="A1:Y43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="26" customWidth="1"/>
@@ -1844,14 +1822,14 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="77"/>
-      <c r="L1" s="77"/>
-      <c r="M1" s="77"/>
-      <c r="N1" s="77"/>
-      <c r="O1" s="77"/>
-      <c r="P1" s="77"/>
-      <c r="Q1" s="77"/>
-      <c r="R1" s="78"/>
+      <c r="K1" s="82"/>
+      <c r="L1" s="82"/>
+      <c r="M1" s="82"/>
+      <c r="N1" s="82"/>
+      <c r="O1" s="82"/>
+      <c r="P1" s="82"/>
+      <c r="Q1" s="82"/>
+      <c r="R1" s="83"/>
     </row>
     <row r="2" spans="1:18" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1861,8 +1839,8 @@
         <v>0</v>
       </c>
       <c r="E2" s="11"/>
-      <c r="F2" s="52" t="s">
-        <v>200</v>
+      <c r="F2" s="51" t="s">
+        <v>195</v>
       </c>
       <c r="G2" s="12"/>
       <c r="H2" s="4"/>
@@ -1885,8 +1863,8 @@
         <v>1</v>
       </c>
       <c r="E3" s="13"/>
-      <c r="F3" s="53" t="s">
-        <v>201</v>
+      <c r="F3" s="52" t="s">
+        <v>196</v>
       </c>
       <c r="G3" s="13"/>
       <c r="H3" s="5"/>
@@ -1899,7 +1877,7 @@
       <c r="O3" s="5"/>
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
-      <c r="R3" s="79"/>
+      <c r="R3" s="84"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1909,8 +1887,8 @@
         <v>2</v>
       </c>
       <c r="E4" s="13"/>
-      <c r="F4" s="54" t="s">
-        <v>201</v>
+      <c r="F4" s="53" t="s">
+        <v>196</v>
       </c>
       <c r="G4" s="14"/>
       <c r="H4" s="7"/>
@@ -1923,7 +1901,7 @@
       <c r="O4" s="6"/>
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
-      <c r="R4" s="80"/>
+      <c r="R4" s="85"/>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1933,7 +1911,7 @@
         <v>3</v>
       </c>
       <c r="E5" s="13"/>
-      <c r="F5" s="55" t="s">
+      <c r="F5" s="54" t="s">
         <v>7</v>
       </c>
       <c r="G5" s="15"/>
@@ -1947,7 +1925,7 @@
       <c r="O5" s="6"/>
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
-      <c r="R5" s="80"/>
+      <c r="R5" s="85"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1967,7 +1945,7 @@
       <c r="O6" s="6"/>
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
-      <c r="R6" s="80"/>
+      <c r="R6" s="85"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1987,7 +1965,7 @@
       <c r="O7" s="8"/>
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
-      <c r="R7" s="80"/>
+      <c r="R7" s="85"/>
     </row>
     <row r="8" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -2007,7 +1985,7 @@
       <c r="O8" s="8"/>
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
-      <c r="R8" s="80"/>
+      <c r="R8" s="85"/>
     </row>
     <row r="9" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -2015,7 +1993,7 @@
         <v>4</v>
       </c>
       <c r="C9" s="30" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="D9" s="30" t="s">
         <v>8</v>
@@ -2023,54 +2001,54 @@
       <c r="E9" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="F9" s="57" t="s">
-        <v>62</v>
+      <c r="F9" s="56" t="s">
+        <v>61</v>
       </c>
       <c r="G9" s="30" t="s">
-        <v>82</v>
-      </c>
-      <c r="H9" s="56" t="s">
-        <v>106</v>
+        <v>81</v>
+      </c>
+      <c r="H9" s="55" t="s">
+        <v>104</v>
       </c>
       <c r="I9" s="30" t="s">
+        <v>139</v>
+      </c>
+      <c r="J9" s="30" t="s">
+        <v>123</v>
+      </c>
+      <c r="K9" s="31" t="s">
+        <v>186</v>
+      </c>
+      <c r="L9" s="30" t="s">
+        <v>137</v>
+      </c>
+      <c r="M9" s="30" t="s">
+        <v>140</v>
+      </c>
+      <c r="N9" s="55" t="s">
+        <v>141</v>
+      </c>
+      <c r="O9" s="30" t="s">
         <v>142</v>
       </c>
-      <c r="J9" s="30" t="s">
-        <v>126</v>
-      </c>
-      <c r="K9" s="31" t="s">
-        <v>191</v>
-      </c>
-      <c r="L9" s="30" t="s">
-        <v>140</v>
-      </c>
-      <c r="M9" s="30" t="s">
+      <c r="P9" s="30" t="s">
         <v>143</v>
       </c>
-      <c r="N9" s="56" t="s">
+      <c r="Q9" s="55" t="s">
         <v>144</v>
       </c>
-      <c r="O9" s="30" t="s">
+      <c r="R9" s="30" t="s">
         <v>145</v>
-      </c>
-      <c r="P9" s="30" t="s">
-        <v>146</v>
-      </c>
-      <c r="Q9" s="56" t="s">
-        <v>147</v>
-      </c>
-      <c r="R9" s="30" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
-      <c r="B10" s="47">
+      <c r="B10" s="46">
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
-      <c r="C10" s="59" t="s">
-        <v>149</v>
+      <c r="C10" s="58" t="s">
+        <v>146</v>
       </c>
       <c r="D10" s="38" t="s">
         <v>9</v>
@@ -2079,24 +2057,24 @@
         <v>34</v>
       </c>
       <c r="F10" s="39" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G10" s="38" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H10" s="39" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="I10" s="38" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="J10" s="39" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="K10" s="38" t="s">
-        <v>128</v>
-      </c>
-      <c r="L10" s="64">
+        <v>125</v>
+      </c>
+      <c r="L10" s="63">
         <v>1</v>
       </c>
       <c r="M10" s="38">
@@ -2106,81 +2084,81 @@
       <c r="N10" s="39">
         <v>40</v>
       </c>
-      <c r="O10" s="62" t="s">
-        <v>197</v>
-      </c>
-      <c r="P10" s="49">
+      <c r="O10" s="61" t="s">
+        <v>192</v>
+      </c>
+      <c r="P10" s="48">
         <v>1.7399999999999999E-2</v>
       </c>
       <c r="Q10" s="40">
         <f>P10*N10</f>
         <v>0.69599999999999995</v>
       </c>
-      <c r="R10" s="85"/>
+      <c r="R10" s="76"/>
     </row>
     <row r="11" spans="1:18" ht="36" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
-      <c r="B11" s="48">
-        <f t="shared" ref="B11:B40" si="0">ROW(B11) - ROW($B$9)</f>
+      <c r="B11" s="47">
+        <f t="shared" ref="B11:B39" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
-      <c r="C11" s="69" t="s">
-        <v>149</v>
-      </c>
-      <c r="D11" s="70" t="s">
-        <v>226</v>
-      </c>
-      <c r="E11" s="70" t="s">
+      <c r="C11" s="68" t="s">
+        <v>146</v>
+      </c>
+      <c r="D11" s="69" t="s">
+        <v>222</v>
+      </c>
+      <c r="E11" s="69" t="s">
         <v>35</v>
       </c>
-      <c r="F11" s="71" t="s">
-        <v>63</v>
-      </c>
-      <c r="G11" s="70" t="s">
-        <v>84</v>
-      </c>
-      <c r="H11" s="71" t="s">
-        <v>107</v>
-      </c>
-      <c r="I11" s="70" t="s">
+      <c r="F11" s="70" t="s">
+        <v>62</v>
+      </c>
+      <c r="G11" s="69" t="s">
+        <v>83</v>
+      </c>
+      <c r="H11" s="70" t="s">
+        <v>105</v>
+      </c>
+      <c r="I11" s="69" t="s">
+        <v>158</v>
+      </c>
+      <c r="J11" s="70" t="s">
         <v>161</v>
       </c>
-      <c r="J11" s="71" t="s">
-        <v>164</v>
-      </c>
-      <c r="K11" s="70" t="s">
-        <v>129</v>
-      </c>
-      <c r="L11" s="73">
-        <v>17</v>
-      </c>
-      <c r="M11" s="70">
+      <c r="K11" s="69" t="s">
+        <v>126</v>
+      </c>
+      <c r="L11" s="72">
+        <v>19</v>
+      </c>
+      <c r="M11" s="69">
         <f t="shared" ref="M11:M41" si="1">L11*20</f>
-        <v>340</v>
-      </c>
-      <c r="N11" s="71">
+        <v>380</v>
+      </c>
+      <c r="N11" s="70">
         <v>400</v>
       </c>
-      <c r="O11" s="63" t="s">
-        <v>197</v>
-      </c>
-      <c r="P11" s="74">
+      <c r="O11" s="62" t="s">
+        <v>192</v>
+      </c>
+      <c r="P11" s="73">
         <v>2.3999999999999998E-3</v>
       </c>
-      <c r="Q11" s="75">
+      <c r="Q11" s="74">
         <f t="shared" ref="Q11" si="2">P11*N11</f>
         <v>0.96</v>
       </c>
-      <c r="R11" s="70"/>
+      <c r="R11" s="69"/>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
-      <c r="B12" s="47">
+      <c r="B12" s="46">
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
-      <c r="C12" s="59" t="s">
-        <v>149</v>
+      <c r="C12" s="58" t="s">
+        <v>146</v>
       </c>
       <c r="D12" s="38" t="s">
         <v>10</v>
@@ -2189,24 +2167,24 @@
         <v>36</v>
       </c>
       <c r="F12" s="39" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="G12" s="38" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H12" s="39" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="I12" s="38" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="J12" s="39" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="K12" s="38" t="s">
-        <v>160</v>
-      </c>
-      <c r="L12" s="64">
+        <v>157</v>
+      </c>
+      <c r="L12" s="63">
         <v>1</v>
       </c>
       <c r="M12" s="38">
@@ -2216,10 +2194,10 @@
       <c r="N12" s="39">
         <v>25</v>
       </c>
-      <c r="O12" s="62" t="s">
-        <v>197</v>
-      </c>
-      <c r="P12" s="49">
+      <c r="O12" s="61" t="s">
+        <v>192</v>
+      </c>
+      <c r="P12" s="48">
         <v>5.2600000000000001E-2</v>
       </c>
       <c r="Q12" s="40">
@@ -2230,67 +2208,67 @@
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
-      <c r="B13" s="48">
+      <c r="B13" s="47">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="69" t="s">
-        <v>149</v>
-      </c>
-      <c r="D13" s="70" t="s">
+      <c r="C13" s="68" t="s">
+        <v>146</v>
+      </c>
+      <c r="D13" s="69" t="s">
         <v>11</v>
       </c>
-      <c r="E13" s="70" t="s">
+      <c r="E13" s="69" t="s">
         <v>37</v>
       </c>
-      <c r="F13" s="71" t="s">
-        <v>64</v>
-      </c>
-      <c r="G13" s="70" t="s">
-        <v>86</v>
-      </c>
-      <c r="H13" s="71" t="s">
-        <v>109</v>
-      </c>
-      <c r="I13" s="70" t="s">
-        <v>161</v>
-      </c>
-      <c r="J13" s="71" t="s">
-        <v>166</v>
-      </c>
-      <c r="K13" s="70" t="s">
-        <v>130</v>
-      </c>
-      <c r="L13" s="73">
+      <c r="F13" s="70" t="s">
+        <v>63</v>
+      </c>
+      <c r="G13" s="69" t="s">
+        <v>85</v>
+      </c>
+      <c r="H13" s="70" t="s">
+        <v>107</v>
+      </c>
+      <c r="I13" s="69" t="s">
+        <v>158</v>
+      </c>
+      <c r="J13" s="70" t="s">
+        <v>163</v>
+      </c>
+      <c r="K13" s="69" t="s">
+        <v>127</v>
+      </c>
+      <c r="L13" s="72">
         <v>2</v>
       </c>
-      <c r="M13" s="70">
+      <c r="M13" s="69">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="N13" s="71">
+      <c r="N13" s="70">
         <v>50</v>
       </c>
-      <c r="O13" s="63" t="s">
-        <v>197</v>
-      </c>
-      <c r="P13" s="74">
+      <c r="O13" s="62" t="s">
+        <v>192</v>
+      </c>
+      <c r="P13" s="73">
         <v>5.96E-2</v>
       </c>
-      <c r="Q13" s="75">
+      <c r="Q13" s="74">
         <f t="shared" ref="Q13" si="3">P13*N13</f>
         <v>2.98</v>
       </c>
-      <c r="R13" s="70"/>
+      <c r="R13" s="69"/>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
-      <c r="B14" s="47">
+      <c r="B14" s="46">
         <f>ROW(B14) - ROW($B$9)</f>
         <v>5</v>
       </c>
-      <c r="C14" s="59" t="s">
-        <v>149</v>
+      <c r="C14" s="58" t="s">
+        <v>146</v>
       </c>
       <c r="D14" s="38" t="s">
         <v>12</v>
@@ -2299,24 +2277,24 @@
         <v>38</v>
       </c>
       <c r="F14" s="39" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G14" s="38" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H14" s="39" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="I14" s="38" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="J14" s="39" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="K14" s="38" t="s">
-        <v>131</v>
-      </c>
-      <c r="L14" s="64">
+        <v>128</v>
+      </c>
+      <c r="L14" s="63">
         <v>2</v>
       </c>
       <c r="M14" s="38">
@@ -2326,10 +2304,10 @@
       <c r="N14" s="39">
         <v>100</v>
       </c>
-      <c r="O14" s="62" t="s">
-        <v>197</v>
-      </c>
-      <c r="P14" s="49">
+      <c r="O14" s="61" t="s">
+        <v>192</v>
+      </c>
+      <c r="P14" s="48">
         <v>2.5999999999999999E-3</v>
       </c>
       <c r="Q14" s="40">
@@ -2340,104 +2318,104 @@
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
-      <c r="B15" s="48">
+      <c r="B15" s="47">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="69" t="s">
-        <v>149</v>
-      </c>
-      <c r="D15" s="70" t="s">
+      <c r="C15" s="68" t="s">
+        <v>146</v>
+      </c>
+      <c r="D15" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="E15" s="70" t="s">
+      <c r="E15" s="69" t="s">
         <v>39</v>
       </c>
-      <c r="F15" s="71" t="s">
-        <v>65</v>
-      </c>
-      <c r="G15" s="72" t="s">
-        <v>88</v>
-      </c>
-      <c r="H15" s="71" t="s">
-        <v>111</v>
-      </c>
-      <c r="I15" s="70" t="s">
-        <v>192</v>
-      </c>
-      <c r="J15" s="71" t="s">
-        <v>168</v>
-      </c>
-      <c r="K15" s="70" t="s">
-        <v>132</v>
-      </c>
-      <c r="L15" s="73">
+      <c r="F15" s="70" t="s">
+        <v>64</v>
+      </c>
+      <c r="G15" s="71" t="s">
+        <v>87</v>
+      </c>
+      <c r="H15" s="70" t="s">
+        <v>109</v>
+      </c>
+      <c r="I15" s="69" t="s">
+        <v>187</v>
+      </c>
+      <c r="J15" s="70" t="s">
+        <v>165</v>
+      </c>
+      <c r="K15" s="69" t="s">
+        <v>129</v>
+      </c>
+      <c r="L15" s="72">
         <v>2</v>
       </c>
-      <c r="M15" s="70">
+      <c r="M15" s="69">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="N15" s="71">
+      <c r="N15" s="70">
         <v>50</v>
       </c>
-      <c r="O15" s="63" t="s">
-        <v>197</v>
-      </c>
-      <c r="P15" s="74">
+      <c r="O15" s="62" t="s">
+        <v>192</v>
+      </c>
+      <c r="P15" s="73">
         <v>6.4000000000000003E-3</v>
       </c>
-      <c r="Q15" s="75">
+      <c r="Q15" s="74">
         <f t="shared" ref="Q15:Q16" si="4">P15*N15</f>
         <v>0.32</v>
       </c>
-      <c r="R15" s="70"/>
+      <c r="R15" s="69"/>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
-      <c r="B16" s="48">
+      <c r="B16" s="47">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C16" s="69" t="s">
-        <v>149</v>
+      <c r="C16" s="68" t="s">
+        <v>146</v>
       </c>
       <c r="D16" s="38" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="E16" s="39" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="F16" s="38" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="G16" s="39" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="H16" s="38" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="I16" s="38"/>
       <c r="J16" s="38" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="K16" s="39" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="L16" s="38">
         <v>1</v>
       </c>
-      <c r="M16" s="70">
+      <c r="M16" s="69">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
       <c r="N16" s="39">
         <v>21</v>
       </c>
-      <c r="O16" s="63" t="s">
-        <v>197</v>
-      </c>
-      <c r="P16" s="49">
+      <c r="O16" s="62" t="s">
+        <v>192</v>
+      </c>
+      <c r="P16" s="48">
         <v>0.46400000000000002</v>
       </c>
       <c r="Q16" s="40">
@@ -2446,14 +2424,14 @@
       </c>
       <c r="R16" s="38"/>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
       <c r="B17" s="47">
-        <f>ROW(B17) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="60" t="s">
-        <v>150</v>
+      <c r="C17" s="59" t="s">
+        <v>147</v>
       </c>
       <c r="D17" s="38" t="s">
         <v>14</v>
@@ -2462,24 +2440,24 @@
         <v>40</v>
       </c>
       <c r="F17" s="39" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G17" s="38" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H17" s="39" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="I17" s="38" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="J17" s="39" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="K17" s="38" t="s">
-        <v>161</v>
-      </c>
-      <c r="L17" s="64">
+        <v>158</v>
+      </c>
+      <c r="L17" s="63">
         <v>1</v>
       </c>
       <c r="M17" s="38">
@@ -2489,10 +2467,10 @@
       <c r="N17" s="39">
         <v>25</v>
       </c>
-      <c r="O17" s="63" t="s">
-        <v>197</v>
-      </c>
-      <c r="P17" s="49">
+      <c r="O17" s="62" t="s">
+        <v>192</v>
+      </c>
+      <c r="P17" s="48">
         <v>6.1699999999999998E-2</v>
       </c>
       <c r="Q17" s="40">
@@ -2501,69 +2479,69 @@
       </c>
       <c r="R17" s="38"/>
     </row>
-    <row r="18" spans="1:22" ht="36" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:25" ht="36" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
-      <c r="B18" s="48">
-        <f t="shared" si="0"/>
+      <c r="B18" s="46">
+        <f>ROW(B18) - ROW($B$9)</f>
         <v>9</v>
       </c>
-      <c r="C18" s="69" t="s">
-        <v>151</v>
-      </c>
-      <c r="D18" s="70" t="s">
+      <c r="C18" s="68" t="s">
+        <v>148</v>
+      </c>
+      <c r="D18" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="E18" s="70" t="s">
+      <c r="E18" s="69" t="s">
         <v>41</v>
       </c>
-      <c r="F18" s="71" t="s">
-        <v>187</v>
-      </c>
-      <c r="G18" s="70" t="s">
-        <v>68</v>
-      </c>
-      <c r="H18" s="71" t="s">
-        <v>111</v>
-      </c>
-      <c r="I18" s="70" t="s">
-        <v>161</v>
-      </c>
-      <c r="J18" s="71" t="s">
-        <v>170</v>
-      </c>
-      <c r="K18" s="70" t="s">
-        <v>161</v>
-      </c>
-      <c r="L18" s="73">
+      <c r="F18" s="70" t="s">
+        <v>183</v>
+      </c>
+      <c r="G18" s="69" t="s">
+        <v>67</v>
+      </c>
+      <c r="H18" s="70" t="s">
+        <v>109</v>
+      </c>
+      <c r="I18" s="69" t="s">
+        <v>158</v>
+      </c>
+      <c r="J18" s="70" t="s">
+        <v>167</v>
+      </c>
+      <c r="K18" s="69" t="s">
+        <v>158</v>
+      </c>
+      <c r="L18" s="72">
         <v>4</v>
       </c>
-      <c r="M18" s="70">
+      <c r="M18" s="69">
         <f t="shared" si="1"/>
         <v>80</v>
       </c>
-      <c r="N18" s="71">
+      <c r="N18" s="70">
         <v>100</v>
       </c>
-      <c r="O18" s="62" t="s">
-        <v>197</v>
-      </c>
-      <c r="P18" s="74">
+      <c r="O18" s="61" t="s">
+        <v>192</v>
+      </c>
+      <c r="P18" s="73">
         <v>2.8000000000000001E-2</v>
       </c>
-      <c r="Q18" s="75">
+      <c r="Q18" s="74">
         <f t="shared" ref="Q18" si="5">P18*N18</f>
         <v>2.8000000000000003</v>
       </c>
-      <c r="R18" s="70"/>
-    </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="R18" s="69"/>
+    </row>
+    <row r="19" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
       <c r="B19" s="47">
-        <f>ROW(B19) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="59" t="s">
-        <v>152</v>
+      <c r="C19" s="58" t="s">
+        <v>149</v>
       </c>
       <c r="D19" s="38" t="s">
         <v>16</v>
@@ -2572,24 +2550,24 @@
         <v>42</v>
       </c>
       <c r="F19" s="39" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="G19" s="38" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="H19" s="39" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="I19" s="38" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="J19" s="39" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="K19" s="38" t="s">
-        <v>161</v>
-      </c>
-      <c r="L19" s="64">
+        <v>158</v>
+      </c>
+      <c r="L19" s="63">
         <v>1</v>
       </c>
       <c r="M19" s="38">
@@ -2599,10 +2577,10 @@
       <c r="N19" s="39">
         <v>22</v>
       </c>
-      <c r="O19" s="63" t="s">
-        <v>198</v>
-      </c>
-      <c r="P19" s="49">
+      <c r="O19" s="62" t="s">
+        <v>193</v>
+      </c>
+      <c r="P19" s="48">
         <v>2.5099999999999998</v>
       </c>
       <c r="Q19" s="40">
@@ -2611,69 +2589,69 @@
       </c>
       <c r="R19" s="38"/>
     </row>
-    <row r="20" spans="1:22" ht="36" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:25" ht="36" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
-      <c r="B20" s="48">
-        <f t="shared" si="0"/>
+      <c r="B20" s="46">
+        <f>ROW(B20) - ROW($B$9)</f>
         <v>11</v>
       </c>
-      <c r="C20" s="69" t="s">
-        <v>151</v>
-      </c>
-      <c r="D20" s="70" t="s">
+      <c r="C20" s="68" t="s">
+        <v>148</v>
+      </c>
+      <c r="D20" s="69" t="s">
         <v>17</v>
       </c>
-      <c r="E20" s="70" t="s">
+      <c r="E20" s="69" t="s">
         <v>43</v>
       </c>
-      <c r="F20" s="71" t="s">
-        <v>70</v>
-      </c>
-      <c r="G20" s="70" t="s">
-        <v>90</v>
-      </c>
-      <c r="H20" s="71" t="s">
-        <v>114</v>
-      </c>
-      <c r="I20" s="70" t="s">
-        <v>161</v>
-      </c>
-      <c r="J20" s="71" t="s">
-        <v>171</v>
-      </c>
-      <c r="K20" s="70" t="s">
-        <v>161</v>
-      </c>
-      <c r="L20" s="73">
+      <c r="F20" s="70" t="s">
+        <v>69</v>
+      </c>
+      <c r="G20" s="69" t="s">
+        <v>89</v>
+      </c>
+      <c r="H20" s="70" t="s">
+        <v>112</v>
+      </c>
+      <c r="I20" s="69" t="s">
+        <v>158</v>
+      </c>
+      <c r="J20" s="70" t="s">
+        <v>168</v>
+      </c>
+      <c r="K20" s="69" t="s">
+        <v>158</v>
+      </c>
+      <c r="L20" s="72">
         <v>1</v>
       </c>
-      <c r="M20" s="70">
+      <c r="M20" s="69">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N20" s="71">
+      <c r="N20" s="70">
         <v>25</v>
       </c>
-      <c r="O20" s="62" t="s">
-        <v>197</v>
-      </c>
-      <c r="P20" s="74">
+      <c r="O20" s="61" t="s">
+        <v>192</v>
+      </c>
+      <c r="P20" s="73">
         <v>8.7599999999999997E-2</v>
       </c>
-      <c r="Q20" s="75">
+      <c r="Q20" s="74">
         <f t="shared" ref="Q20" si="6">P20*N20</f>
         <v>2.19</v>
       </c>
-      <c r="R20" s="70"/>
-    </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="R20" s="69"/>
+    </row>
+    <row r="21" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
       <c r="B21" s="47">
-        <f>ROW(B21) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C21" s="59" t="s">
-        <v>153</v>
+      <c r="C21" s="58" t="s">
+        <v>150</v>
       </c>
       <c r="D21" s="38" t="s">
         <v>18</v>
@@ -2682,24 +2660,24 @@
         <v>44</v>
       </c>
       <c r="F21" s="39" t="s">
-        <v>71</v>
-      </c>
-      <c r="G21" s="61" t="s">
-        <v>91</v>
+        <v>70</v>
+      </c>
+      <c r="G21" s="60" t="s">
+        <v>90</v>
       </c>
       <c r="H21" s="39" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="I21" s="38" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="J21" s="39" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="K21" s="38" t="s">
-        <v>161</v>
-      </c>
-      <c r="L21" s="64">
+        <v>158</v>
+      </c>
+      <c r="L21" s="63">
         <v>1</v>
       </c>
       <c r="M21" s="38">
@@ -2709,10 +2687,10 @@
       <c r="N21" s="39">
         <v>30</v>
       </c>
-      <c r="O21" s="63" t="s">
-        <v>197</v>
-      </c>
-      <c r="P21" s="49">
+      <c r="O21" s="62" t="s">
+        <v>192</v>
+      </c>
+      <c r="P21" s="48">
         <v>3.7900000000000003E-2</v>
       </c>
       <c r="Q21" s="40">
@@ -2721,126 +2699,125 @@
       </c>
       <c r="R21" s="38"/>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
-      <c r="B22" s="48">
+      <c r="B22" s="47">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C22" s="69" t="s">
-        <v>154</v>
-      </c>
-      <c r="D22" s="70" t="s">
+      <c r="C22" s="68" t="s">
+        <v>151</v>
+      </c>
+      <c r="D22" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="E22" s="70" t="s">
+      <c r="E22" s="69" t="s">
         <v>45</v>
       </c>
-      <c r="F22" s="71" t="s">
-        <v>186</v>
-      </c>
-      <c r="G22" s="70" t="s">
-        <v>72</v>
-      </c>
-      <c r="H22" s="71" t="s">
-        <v>116</v>
-      </c>
-      <c r="I22" s="70" t="s">
-        <v>161</v>
-      </c>
-      <c r="J22" s="71" t="s">
-        <v>161</v>
-      </c>
-      <c r="K22" s="70" t="s">
-        <v>161</v>
-      </c>
-      <c r="L22" s="73">
+      <c r="F22" s="70" t="s">
+        <v>182</v>
+      </c>
+      <c r="G22" s="69" t="s">
+        <v>71</v>
+      </c>
+      <c r="H22" s="70" t="s">
+        <v>114</v>
+      </c>
+      <c r="I22" s="69" t="s">
+        <v>158</v>
+      </c>
+      <c r="J22" s="70" t="s">
+        <v>158</v>
+      </c>
+      <c r="K22" s="69" t="s">
+        <v>158</v>
+      </c>
+      <c r="L22" s="72">
         <v>1</v>
       </c>
-      <c r="M22" s="70">
+      <c r="M22" s="69">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N22" s="71">
+      <c r="N22" s="70">
         <v>25</v>
       </c>
-      <c r="O22" s="62" t="s">
-        <v>199</v>
-      </c>
-      <c r="P22" s="74">
+      <c r="O22" s="61" t="s">
+        <v>194</v>
+      </c>
+      <c r="P22" s="73">
         <v>0.30840000000000001</v>
       </c>
-      <c r="Q22" s="75">
+      <c r="Q22" s="74">
         <f t="shared" ref="Q22" si="7">P22*N22</f>
         <v>7.71</v>
       </c>
-      <c r="R22" s="70"/>
-    </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="R22" s="69"/>
+    </row>
+    <row r="23" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
-      <c r="B23" s="48">
-        <f t="shared" si="0"/>
+      <c r="B23" s="46">
+        <f>ROW(B23) - ROW($B$9)</f>
         <v>14</v>
       </c>
-      <c r="C23" s="87" t="s">
-        <v>217</v>
-      </c>
-      <c r="D23" s="72" t="s">
-        <v>208</v>
-      </c>
-      <c r="E23" s="72" t="s">
-        <v>218</v>
-      </c>
-      <c r="F23" s="72" t="s">
-        <v>205</v>
-      </c>
-      <c r="G23" s="72" t="s">
-        <v>205</v>
-      </c>
-      <c r="H23" s="72" t="s">
-        <v>161</v>
-      </c>
-      <c r="I23" s="72" t="s">
-        <v>161</v>
-      </c>
-      <c r="J23" s="72" t="s">
-        <v>161</v>
-      </c>
-      <c r="K23" s="72" t="s">
-        <v>219</v>
-      </c>
-      <c r="L23" s="72">
+      <c r="C23" s="78" t="s">
+        <v>212</v>
+      </c>
+      <c r="D23" s="71" t="s">
+        <v>203</v>
+      </c>
+      <c r="E23" s="71" t="s">
+        <v>213</v>
+      </c>
+      <c r="F23" s="71" t="s">
+        <v>200</v>
+      </c>
+      <c r="G23" s="71" t="s">
+        <v>200</v>
+      </c>
+      <c r="H23" s="71" t="s">
+        <v>158</v>
+      </c>
+      <c r="I23" s="71" t="s">
+        <v>158</v>
+      </c>
+      <c r="J23" s="71" t="s">
+        <v>158</v>
+      </c>
+      <c r="K23" s="71" t="s">
+        <v>214</v>
+      </c>
+      <c r="L23" s="71">
         <v>6</v>
       </c>
-      <c r="M23" s="72">
+      <c r="M23" s="71">
         <f t="shared" si="1"/>
         <v>120</v>
       </c>
-      <c r="N23" s="72" t="s">
-        <v>161</v>
-      </c>
-      <c r="O23" s="72" t="s">
-        <v>161</v>
-      </c>
-      <c r="P23" s="89" t="s">
-        <v>161</v>
-      </c>
-      <c r="Q23" s="89" t="s">
-        <v>161</v>
-      </c>
-      <c r="R23" s="72" t="s">
-        <v>220</v>
-      </c>
-      <c r="S23" s="88"/>
-    </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A24" s="1"/>
+      <c r="N23" s="71" t="s">
+        <v>158</v>
+      </c>
+      <c r="O23" s="71" t="s">
+        <v>158</v>
+      </c>
+      <c r="P23" s="79" t="s">
+        <v>158</v>
+      </c>
+      <c r="Q23" s="79" t="s">
+        <v>158</v>
+      </c>
+      <c r="R23" s="71" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="24" spans="1:25" s="81" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="80"/>
       <c r="B24" s="47">
-        <f>ROW(B24) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C24" s="59" t="s">
-        <v>155</v>
+      <c r="C24" s="58" t="s">
+        <v>152</v>
       </c>
       <c r="D24" s="38" t="s">
         <v>20</v>
@@ -2849,24 +2826,24 @@
         <v>46</v>
       </c>
       <c r="F24" s="39" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G24" s="38" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H24" s="39" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="I24" s="38" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="J24" s="39" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="K24" s="38" t="s">
-        <v>161</v>
-      </c>
-      <c r="L24" s="64">
+        <v>158</v>
+      </c>
+      <c r="L24" s="63">
         <v>2</v>
       </c>
       <c r="M24" s="38">
@@ -2876,10 +2853,10 @@
       <c r="N24" s="39">
         <v>60</v>
       </c>
-      <c r="O24" s="63" t="s">
-        <v>197</v>
-      </c>
-      <c r="P24" s="49">
+      <c r="O24" s="62" t="s">
+        <v>192</v>
+      </c>
+      <c r="P24" s="48">
         <v>3.0599999999999999E-2</v>
       </c>
       <c r="Q24" s="40">
@@ -2887,73 +2864,76 @@
         <v>1.8359999999999999</v>
       </c>
       <c r="R24" s="38"/>
-    </row>
-    <row r="25" spans="1:22" s="91" customFormat="1" ht="72" x14ac:dyDescent="0.25">
-      <c r="A25" s="90"/>
-      <c r="B25" s="48">
-        <f t="shared" si="0"/>
+      <c r="T24"/>
+      <c r="U24"/>
+      <c r="V24"/>
+      <c r="W24"/>
+      <c r="X24"/>
+      <c r="Y24"/>
+    </row>
+    <row r="25" spans="1:25" ht="72" x14ac:dyDescent="0.25">
+      <c r="A25" s="1"/>
+      <c r="B25" s="46">
+        <f>ROW(B25) - ROW($B$9)</f>
         <v>16</v>
       </c>
-      <c r="C25" s="69" t="s">
-        <v>156</v>
-      </c>
-      <c r="D25" s="70" t="s">
-        <v>209</v>
-      </c>
-      <c r="E25" s="70" t="s">
+      <c r="C25" s="68" t="s">
+        <v>153</v>
+      </c>
+      <c r="D25" s="69" t="s">
+        <v>204</v>
+      </c>
+      <c r="E25" s="69" t="s">
         <v>47</v>
       </c>
-      <c r="F25" s="71" t="s">
-        <v>73</v>
-      </c>
-      <c r="G25" s="70" t="s">
-        <v>93</v>
-      </c>
-      <c r="H25" s="71" t="s">
-        <v>110</v>
-      </c>
-      <c r="I25" s="70" t="s">
-        <v>161</v>
-      </c>
-      <c r="J25" s="71" t="s">
-        <v>174</v>
-      </c>
-      <c r="K25" s="70" t="s">
-        <v>133</v>
-      </c>
-      <c r="L25" s="70">
+      <c r="F25" s="70" t="s">
+        <v>72</v>
+      </c>
+      <c r="G25" s="69" t="s">
+        <v>92</v>
+      </c>
+      <c r="H25" s="70" t="s">
+        <v>108</v>
+      </c>
+      <c r="I25" s="69" t="s">
+        <v>158</v>
+      </c>
+      <c r="J25" s="70" t="s">
+        <v>171</v>
+      </c>
+      <c r="K25" s="69" t="s">
+        <v>130</v>
+      </c>
+      <c r="L25" s="69">
         <v>38</v>
       </c>
-      <c r="M25" s="70">
+      <c r="M25" s="69">
         <f t="shared" si="1"/>
         <v>760</v>
       </c>
-      <c r="N25" s="71">
+      <c r="N25" s="70">
         <v>800</v>
       </c>
-      <c r="O25" s="62" t="s">
-        <v>197</v>
-      </c>
-      <c r="P25" s="74">
+      <c r="O25" s="61" t="s">
+        <v>192</v>
+      </c>
+      <c r="P25" s="73">
         <v>8.0000000000000004E-4</v>
       </c>
-      <c r="Q25" s="75">
+      <c r="Q25" s="74">
         <f t="shared" ref="Q25" si="8">P25*N25</f>
         <v>0.64</v>
       </c>
-      <c r="R25" s="70"/>
-      <c r="T25"/>
-      <c r="U25"/>
-      <c r="V25"/>
-    </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="R25" s="69"/>
+    </row>
+    <row r="26" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
       <c r="B26" s="47">
-        <f>ROW(B26) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="C26" s="59" t="s">
-        <v>156</v>
+      <c r="C26" s="58" t="s">
+        <v>153</v>
       </c>
       <c r="D26" s="38" t="s">
         <v>21</v>
@@ -2962,24 +2942,24 @@
         <v>48</v>
       </c>
       <c r="F26" s="39" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G26" s="38" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H26" s="39" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="I26" s="38" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="J26" s="39" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="K26" s="38" t="s">
-        <v>134</v>
-      </c>
-      <c r="L26" s="64">
+        <v>131</v>
+      </c>
+      <c r="L26" s="63">
         <v>7</v>
       </c>
       <c r="M26" s="38">
@@ -2989,10 +2969,10 @@
       <c r="N26" s="39">
         <v>200</v>
       </c>
-      <c r="O26" s="63" t="s">
-        <v>197</v>
-      </c>
-      <c r="P26" s="49">
+      <c r="O26" s="62" t="s">
+        <v>192</v>
+      </c>
+      <c r="P26" s="48">
         <v>1E-3</v>
       </c>
       <c r="Q26" s="40">
@@ -3001,69 +2981,69 @@
       </c>
       <c r="R26" s="38"/>
     </row>
-    <row r="27" spans="1:22" ht="36" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:25" ht="36" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
-      <c r="B27" s="48">
-        <f t="shared" si="0"/>
+      <c r="B27" s="46">
+        <f>ROW(B27) - ROW($B$9)</f>
         <v>18</v>
       </c>
-      <c r="C27" s="69" t="s">
-        <v>156</v>
-      </c>
-      <c r="D27" s="70" t="s">
+      <c r="C27" s="68" t="s">
+        <v>153</v>
+      </c>
+      <c r="D27" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="E27" s="70" t="s">
+      <c r="E27" s="69" t="s">
         <v>49</v>
       </c>
-      <c r="F27" s="71" t="s">
-        <v>73</v>
-      </c>
-      <c r="G27" s="72" t="s">
-        <v>95</v>
-      </c>
-      <c r="H27" s="71" t="s">
-        <v>118</v>
-      </c>
-      <c r="I27" s="70" t="s">
-        <v>194</v>
-      </c>
-      <c r="J27" s="71" t="s">
-        <v>176</v>
-      </c>
-      <c r="K27" s="70" t="s">
-        <v>135</v>
-      </c>
-      <c r="L27" s="73">
+      <c r="F27" s="70" t="s">
+        <v>72</v>
+      </c>
+      <c r="G27" s="71" t="s">
+        <v>94</v>
+      </c>
+      <c r="H27" s="70" t="s">
+        <v>116</v>
+      </c>
+      <c r="I27" s="69" t="s">
+        <v>189</v>
+      </c>
+      <c r="J27" s="70" t="s">
+        <v>173</v>
+      </c>
+      <c r="K27" s="69" t="s">
+        <v>132</v>
+      </c>
+      <c r="L27" s="72">
         <v>1</v>
       </c>
-      <c r="M27" s="70">
+      <c r="M27" s="69">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N27" s="71">
+      <c r="N27" s="70">
         <v>100</v>
       </c>
-      <c r="O27" s="62" t="s">
-        <v>197</v>
-      </c>
-      <c r="P27" s="74">
+      <c r="O27" s="61" t="s">
+        <v>192</v>
+      </c>
+      <c r="P27" s="73">
         <v>1.9E-3</v>
       </c>
-      <c r="Q27" s="75">
+      <c r="Q27" s="74">
         <f t="shared" ref="Q27" si="9">P27*N27</f>
         <v>0.19</v>
       </c>
-      <c r="R27" s="70"/>
-    </row>
-    <row r="28" spans="1:22" ht="24" x14ac:dyDescent="0.25">
+      <c r="R27" s="69"/>
+    </row>
+    <row r="28" spans="1:25" ht="24" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
       <c r="B28" s="47">
-        <f>ROW(B28) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="C28" s="59" t="s">
-        <v>156</v>
+      <c r="C28" s="58" t="s">
+        <v>153</v>
       </c>
       <c r="D28" s="38" t="s">
         <v>23</v>
@@ -3072,24 +3052,24 @@
         <v>50</v>
       </c>
       <c r="F28" s="39" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G28" s="38" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H28" s="39" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="I28" s="38" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="J28" s="39" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="K28" s="38" t="s">
-        <v>136</v>
-      </c>
-      <c r="L28" s="64">
+        <v>133</v>
+      </c>
+      <c r="L28" s="63">
         <v>2</v>
       </c>
       <c r="M28" s="38">
@@ -3099,10 +3079,10 @@
       <c r="N28" s="39">
         <v>100</v>
       </c>
-      <c r="O28" s="63" t="s">
-        <v>197</v>
-      </c>
-      <c r="P28" s="49">
+      <c r="O28" s="62" t="s">
+        <v>192</v>
+      </c>
+      <c r="P28" s="48">
         <v>1E-3</v>
       </c>
       <c r="Q28" s="40">
@@ -3111,69 +3091,69 @@
       </c>
       <c r="R28" s="38"/>
     </row>
-    <row r="29" spans="1:22" ht="24" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:25" ht="24" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
-      <c r="B29" s="48">
-        <f t="shared" si="0"/>
+      <c r="B29" s="46">
+        <f>ROW(B29) - ROW($B$9)</f>
         <v>20</v>
       </c>
-      <c r="C29" s="69" t="s">
-        <v>156</v>
-      </c>
-      <c r="D29" s="70" t="s">
-        <v>210</v>
-      </c>
-      <c r="E29" s="70" t="s">
-        <v>221</v>
-      </c>
-      <c r="F29" s="71" t="s">
-        <v>74</v>
-      </c>
-      <c r="G29" s="70" t="s">
-        <v>97</v>
-      </c>
-      <c r="H29" s="71" t="s">
-        <v>110</v>
-      </c>
-      <c r="I29" s="70" t="s">
-        <v>161</v>
-      </c>
-      <c r="J29" s="71" t="s">
-        <v>178</v>
-      </c>
-      <c r="K29" s="70" t="s">
-        <v>137</v>
-      </c>
-      <c r="L29" s="73">
+      <c r="C29" s="68" t="s">
+        <v>153</v>
+      </c>
+      <c r="D29" s="69" t="s">
+        <v>205</v>
+      </c>
+      <c r="E29" s="69" t="s">
+        <v>216</v>
+      </c>
+      <c r="F29" s="70" t="s">
+        <v>73</v>
+      </c>
+      <c r="G29" s="69" t="s">
+        <v>96</v>
+      </c>
+      <c r="H29" s="70" t="s">
+        <v>108</v>
+      </c>
+      <c r="I29" s="69" t="s">
+        <v>158</v>
+      </c>
+      <c r="J29" s="70" t="s">
+        <v>175</v>
+      </c>
+      <c r="K29" s="69" t="s">
+        <v>134</v>
+      </c>
+      <c r="L29" s="72">
         <v>1</v>
       </c>
-      <c r="M29" s="70">
+      <c r="M29" s="69">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N29" s="71">
+      <c r="N29" s="70">
         <v>100</v>
       </c>
-      <c r="O29" s="62" t="s">
-        <v>197</v>
-      </c>
-      <c r="P29" s="74">
+      <c r="O29" s="61" t="s">
+        <v>192</v>
+      </c>
+      <c r="P29" s="73">
         <v>1.2999999999999999E-3</v>
       </c>
-      <c r="Q29" s="75">
+      <c r="Q29" s="74">
         <f t="shared" ref="Q29" si="10">P29*N29</f>
         <v>0.13</v>
       </c>
-      <c r="R29" s="70"/>
-    </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="R29" s="69"/>
+    </row>
+    <row r="30" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
       <c r="B30" s="47">
-        <f>ROW(B30) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="C30" s="59" t="s">
-        <v>156</v>
+      <c r="C30" s="58" t="s">
+        <v>153</v>
       </c>
       <c r="D30" s="38" t="s">
         <v>24</v>
@@ -3182,24 +3162,24 @@
         <v>51</v>
       </c>
       <c r="F30" s="39" t="s">
-        <v>74</v>
-      </c>
-      <c r="G30" s="61" t="s">
-        <v>98</v>
+        <v>73</v>
+      </c>
+      <c r="G30" s="60" t="s">
+        <v>97</v>
       </c>
       <c r="H30" s="39" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="I30" s="38" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="J30" s="39" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="K30" s="38" t="s">
-        <v>138</v>
-      </c>
-      <c r="L30" s="64">
+        <v>135</v>
+      </c>
+      <c r="L30" s="63">
         <v>2</v>
       </c>
       <c r="M30" s="38">
@@ -3209,10 +3189,10 @@
       <c r="N30" s="39">
         <v>50</v>
       </c>
-      <c r="O30" s="63" t="s">
-        <v>197</v>
-      </c>
-      <c r="P30" s="49">
+      <c r="O30" s="62" t="s">
+        <v>192</v>
+      </c>
+      <c r="P30" s="48">
         <v>2.7000000000000001E-3</v>
       </c>
       <c r="Q30" s="40">
@@ -3221,124 +3201,124 @@
       </c>
       <c r="R30" s="38"/>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
-      <c r="B31" s="48">
+      <c r="B31" s="47">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="C31" s="69" t="s">
-        <v>156</v>
-      </c>
-      <c r="D31" s="70" t="s">
-        <v>211</v>
-      </c>
-      <c r="E31" s="70" t="s">
-        <v>222</v>
-      </c>
-      <c r="F31" s="70" t="s">
-        <v>223</v>
-      </c>
-      <c r="G31" s="70" t="s">
+      <c r="C31" s="68" t="s">
+        <v>153</v>
+      </c>
+      <c r="D31" s="69" t="s">
         <v>206</v>
       </c>
-      <c r="H31" s="70" t="s">
-        <v>110</v>
-      </c>
-      <c r="I31" s="70" t="s">
-        <v>161</v>
-      </c>
-      <c r="J31" s="70" t="s">
-        <v>224</v>
-      </c>
-      <c r="K31" s="70" t="s">
-        <v>225</v>
-      </c>
-      <c r="L31" s="70">
+      <c r="E31" s="69" t="s">
+        <v>217</v>
+      </c>
+      <c r="F31" s="69" t="s">
+        <v>218</v>
+      </c>
+      <c r="G31" s="69" t="s">
+        <v>201</v>
+      </c>
+      <c r="H31" s="69" t="s">
+        <v>108</v>
+      </c>
+      <c r="I31" s="69" t="s">
+        <v>158</v>
+      </c>
+      <c r="J31" s="69" t="s">
+        <v>219</v>
+      </c>
+      <c r="K31" s="69" t="s">
+        <v>220</v>
+      </c>
+      <c r="L31" s="69">
         <v>4</v>
       </c>
-      <c r="M31" s="70">
-        <f t="shared" ref="M31" si="11">L31*5</f>
-        <v>20</v>
-      </c>
-      <c r="N31" s="70">
+      <c r="M31" s="38">
+        <f t="shared" si="1"/>
+        <v>80</v>
+      </c>
+      <c r="N31" s="69">
         <v>100</v>
       </c>
-      <c r="O31" s="63" t="s">
-        <v>197</v>
-      </c>
-      <c r="P31" s="75">
+      <c r="O31" s="62" t="s">
+        <v>192</v>
+      </c>
+      <c r="P31" s="74">
         <v>1.1999999999999999E-3</v>
       </c>
-      <c r="Q31" s="75">
-        <f t="shared" ref="Q31" si="12">P31*N31</f>
+      <c r="Q31" s="74">
+        <f t="shared" ref="Q31" si="11">P31*N31</f>
         <v>0.12</v>
       </c>
-      <c r="R31" s="70"/>
-    </row>
-    <row r="32" spans="1:22" ht="60" x14ac:dyDescent="0.25">
+      <c r="R31" s="69"/>
+    </row>
+    <row r="32" spans="1:25" ht="60" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
-      <c r="B32" s="48">
-        <f t="shared" si="0"/>
+      <c r="B32" s="46">
+        <f>ROW(B32) - ROW($B$9)</f>
         <v>23</v>
       </c>
-      <c r="C32" s="69" t="s">
-        <v>157</v>
-      </c>
-      <c r="D32" s="70" t="s">
+      <c r="C32" s="68" t="s">
+        <v>154</v>
+      </c>
+      <c r="D32" s="69" t="s">
         <v>25</v>
       </c>
-      <c r="E32" s="70" t="s">
+      <c r="E32" s="69" t="s">
         <v>52</v>
       </c>
-      <c r="F32" s="71" t="s">
-        <v>186</v>
-      </c>
-      <c r="G32" s="70" t="s">
-        <v>75</v>
-      </c>
-      <c r="H32" s="71" t="s">
-        <v>119</v>
-      </c>
-      <c r="I32" s="70" t="s">
-        <v>161</v>
-      </c>
-      <c r="J32" s="71" t="s">
-        <v>180</v>
-      </c>
-      <c r="K32" s="70" t="s">
-        <v>161</v>
-      </c>
-      <c r="L32" s="73">
+      <c r="F32" s="70" t="s">
+        <v>182</v>
+      </c>
+      <c r="G32" s="69" t="s">
+        <v>74</v>
+      </c>
+      <c r="H32" s="70" t="s">
+        <v>117</v>
+      </c>
+      <c r="I32" s="69" t="s">
+        <v>158</v>
+      </c>
+      <c r="J32" s="70" t="s">
+        <v>177</v>
+      </c>
+      <c r="K32" s="69" t="s">
+        <v>158</v>
+      </c>
+      <c r="L32" s="72">
         <v>1</v>
       </c>
-      <c r="M32" s="70">
+      <c r="M32" s="69">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N32" s="71">
+      <c r="N32" s="70">
         <v>30</v>
       </c>
-      <c r="O32" s="63" t="s">
-        <v>197</v>
-      </c>
-      <c r="P32" s="74">
+      <c r="O32" s="62" t="s">
+        <v>192</v>
+      </c>
+      <c r="P32" s="73">
         <v>4.1399999999999999E-2</v>
       </c>
-      <c r="Q32" s="75">
-        <f t="shared" ref="Q32" si="13">P32*N32</f>
+      <c r="Q32" s="74">
+        <f t="shared" ref="Q32" si="12">P32*N32</f>
         <v>1.242</v>
       </c>
-      <c r="R32" s="70"/>
+      <c r="R32" s="69"/>
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
       <c r="B33" s="47">
-        <f>ROW(B33) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="C33" s="59" t="s">
-        <v>158</v>
+      <c r="C33" s="58" t="s">
+        <v>155</v>
       </c>
       <c r="D33" s="38" t="s">
         <v>26</v>
@@ -3347,24 +3327,24 @@
         <v>53</v>
       </c>
       <c r="F33" s="39" t="s">
-        <v>188</v>
-      </c>
-      <c r="G33" s="61" t="s">
-        <v>99</v>
+        <v>184</v>
+      </c>
+      <c r="G33" s="60" t="s">
+        <v>98</v>
       </c>
       <c r="H33" s="39" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="I33" s="38" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="J33" s="39" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="K33" s="38" t="s">
-        <v>161</v>
-      </c>
-      <c r="L33" s="64">
+        <v>158</v>
+      </c>
+      <c r="L33" s="63">
         <v>1</v>
       </c>
       <c r="M33" s="38">
@@ -3374,219 +3354,219 @@
       <c r="N33" s="39">
         <v>22</v>
       </c>
-      <c r="O33" s="62" t="s">
-        <v>197</v>
-      </c>
-      <c r="P33" s="49">
+      <c r="O33" s="61" t="s">
+        <v>192</v>
+      </c>
+      <c r="P33" s="48">
         <v>10.652799999999999</v>
       </c>
       <c r="Q33" s="40">
         <f>P33*N33</f>
         <v>234.36159999999998</v>
       </c>
-      <c r="R33" s="76" t="s">
-        <v>202</v>
+      <c r="R33" s="75" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
-      <c r="B34" s="48">
-        <f t="shared" si="0"/>
+      <c r="B34" s="46">
+        <f>ROW(B34) - ROW($B$9)</f>
         <v>25</v>
       </c>
-      <c r="C34" s="69" t="s">
-        <v>158</v>
-      </c>
-      <c r="D34" s="70" t="s">
+      <c r="C34" s="68" t="s">
+        <v>155</v>
+      </c>
+      <c r="D34" s="69" t="s">
         <v>27</v>
       </c>
-      <c r="E34" s="70" t="s">
+      <c r="E34" s="69" t="s">
         <v>54</v>
       </c>
-      <c r="F34" s="71" t="s">
-        <v>76</v>
-      </c>
-      <c r="G34" s="86" t="s">
-        <v>100</v>
-      </c>
-      <c r="H34" s="71" t="s">
-        <v>121</v>
-      </c>
-      <c r="I34" s="70" t="s">
-        <v>161</v>
-      </c>
-      <c r="J34" s="71" t="s">
-        <v>182</v>
-      </c>
-      <c r="K34" s="70" t="s">
-        <v>161</v>
-      </c>
-      <c r="L34" s="73">
+      <c r="F34" s="70" t="s">
+        <v>75</v>
+      </c>
+      <c r="G34" s="77" t="s">
+        <v>99</v>
+      </c>
+      <c r="H34" s="70" t="s">
+        <v>119</v>
+      </c>
+      <c r="I34" s="69" t="s">
+        <v>158</v>
+      </c>
+      <c r="J34" s="70" t="s">
+        <v>179</v>
+      </c>
+      <c r="K34" s="69" t="s">
+        <v>158</v>
+      </c>
+      <c r="L34" s="72">
         <v>1</v>
       </c>
-      <c r="M34" s="70">
+      <c r="M34" s="69">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N34" s="71">
+      <c r="N34" s="70">
         <v>22</v>
       </c>
-      <c r="O34" s="63" t="s">
-        <v>197</v>
-      </c>
-      <c r="P34" s="74">
+      <c r="O34" s="62" t="s">
+        <v>192</v>
+      </c>
+      <c r="P34" s="73">
         <v>1.6387</v>
       </c>
-      <c r="Q34" s="75">
-        <f t="shared" ref="Q34" si="14">P34*N34</f>
+      <c r="Q34" s="74">
+        <f t="shared" ref="Q34:Q35" si="13">P34*N34</f>
         <v>36.051400000000001</v>
       </c>
-      <c r="R34" s="70"/>
+      <c r="R34" s="69"/>
     </row>
     <row r="35" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
       <c r="B35" s="47">
-        <f>ROW(B35) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="C35" s="59" t="s">
-        <v>158</v>
-      </c>
-      <c r="D35" s="38" t="s">
+      <c r="C35" s="78" t="s">
+        <v>155</v>
+      </c>
+      <c r="D35" s="69" t="s">
         <v>28</v>
       </c>
-      <c r="E35" s="38" t="s">
-        <v>55</v>
-      </c>
-      <c r="F35" s="39" t="s">
-        <v>189</v>
-      </c>
-      <c r="G35" s="61" t="s">
-        <v>101</v>
-      </c>
-      <c r="H35" s="39" t="s">
-        <v>122</v>
-      </c>
-      <c r="I35" s="38" t="s">
-        <v>101</v>
-      </c>
-      <c r="J35" s="39" t="s">
-        <v>183</v>
-      </c>
-      <c r="K35" s="38" t="s">
-        <v>161</v>
-      </c>
-      <c r="L35" s="64">
+      <c r="E35" s="69" t="s">
+        <v>223</v>
+      </c>
+      <c r="F35" s="69" t="s">
+        <v>224</v>
+      </c>
+      <c r="G35" s="69" t="s">
+        <v>221</v>
+      </c>
+      <c r="H35" s="69" t="s">
+        <v>225</v>
+      </c>
+      <c r="I35" s="69" t="s">
+        <v>158</v>
+      </c>
+      <c r="J35" s="69" t="s">
+        <v>158</v>
+      </c>
+      <c r="K35" s="69" t="s">
+        <v>158</v>
+      </c>
+      <c r="L35" s="69">
         <v>1</v>
       </c>
-      <c r="M35" s="38">
+      <c r="M35" s="69">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N35" s="39">
-        <v>22</v>
-      </c>
-      <c r="O35" s="62" t="s">
-        <v>197</v>
-      </c>
-      <c r="P35" s="49">
-        <v>3.0720999999999998</v>
-      </c>
-      <c r="Q35" s="40">
-        <f>P35*N35</f>
-        <v>67.586199999999991</v>
+      <c r="N35" s="69">
+        <v>21</v>
+      </c>
+      <c r="O35" s="90" t="s">
+        <v>194</v>
+      </c>
+      <c r="P35" s="74">
+        <v>21.32</v>
+      </c>
+      <c r="Q35" s="74">
+        <f t="shared" si="13"/>
+        <v>447.72</v>
       </c>
       <c r="R35" s="38"/>
     </row>
     <row r="36" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
-      <c r="B36" s="48">
-        <f t="shared" si="0"/>
+      <c r="B36" s="46">
+        <f>ROW(B36) - ROW($B$9)</f>
         <v>27</v>
       </c>
-      <c r="C36" s="69" t="s">
-        <v>158</v>
-      </c>
-      <c r="D36" s="70" t="s">
+      <c r="C36" s="68" t="s">
+        <v>155</v>
+      </c>
+      <c r="D36" s="69" t="s">
         <v>29</v>
       </c>
-      <c r="E36" s="70" t="s">
-        <v>56</v>
-      </c>
-      <c r="F36" s="71" t="s">
-        <v>190</v>
-      </c>
-      <c r="G36" s="72" t="s">
-        <v>102</v>
-      </c>
-      <c r="H36" s="71" t="s">
-        <v>120</v>
-      </c>
-      <c r="I36" s="70" t="s">
-        <v>102</v>
-      </c>
-      <c r="J36" s="71" t="s">
-        <v>127</v>
-      </c>
-      <c r="K36" s="70" t="s">
-        <v>161</v>
-      </c>
-      <c r="L36" s="73">
+      <c r="E36" s="69" t="s">
+        <v>55</v>
+      </c>
+      <c r="F36" s="70" t="s">
+        <v>185</v>
+      </c>
+      <c r="G36" s="71" t="s">
+        <v>100</v>
+      </c>
+      <c r="H36" s="70" t="s">
+        <v>118</v>
+      </c>
+      <c r="I36" s="69" t="s">
+        <v>100</v>
+      </c>
+      <c r="J36" s="70" t="s">
+        <v>124</v>
+      </c>
+      <c r="K36" s="69" t="s">
+        <v>158</v>
+      </c>
+      <c r="L36" s="72">
         <v>1</v>
       </c>
-      <c r="M36" s="70">
+      <c r="M36" s="69">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N36" s="71">
+      <c r="N36" s="70">
         <v>22</v>
       </c>
-      <c r="O36" s="63" t="s">
-        <v>197</v>
-      </c>
-      <c r="P36" s="74">
+      <c r="O36" s="62" t="s">
+        <v>192</v>
+      </c>
+      <c r="P36" s="73">
         <v>1.8360000000000001</v>
       </c>
-      <c r="Q36" s="75">
-        <f t="shared" ref="Q36" si="15">P36*N36</f>
+      <c r="Q36" s="74">
+        <f t="shared" ref="Q36" si="14">P36*N36</f>
         <v>40.392000000000003</v>
       </c>
-      <c r="R36" s="70"/>
+      <c r="R36" s="69"/>
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A37" s="1"/>
       <c r="B37" s="47">
-        <f>ROW(B37) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="C37" s="59" t="s">
-        <v>158</v>
+      <c r="C37" s="58" t="s">
+        <v>155</v>
       </c>
       <c r="D37" s="38" t="s">
         <v>30</v>
       </c>
       <c r="E37" s="38" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F37" s="39" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G37" s="38" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="H37" s="39" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="I37" s="38" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="J37" s="39" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="K37" s="38" t="s">
-        <v>161</v>
-      </c>
-      <c r="L37" s="64">
+        <v>158</v>
+      </c>
+      <c r="L37" s="63">
         <v>1</v>
       </c>
       <c r="M37" s="38">
@@ -3596,10 +3576,10 @@
       <c r="N37" s="39">
         <v>25</v>
       </c>
-      <c r="O37" s="62" t="s">
-        <v>197</v>
-      </c>
-      <c r="P37" s="49">
+      <c r="O37" s="61" t="s">
+        <v>192</v>
+      </c>
+      <c r="P37" s="48">
         <v>0.22670000000000001</v>
       </c>
       <c r="Q37" s="40">
@@ -3610,93 +3590,93 @@
     </row>
     <row r="38" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
-      <c r="B38" s="48">
-        <f t="shared" si="0"/>
+      <c r="B38" s="46">
+        <f>ROW(B38) - ROW($B$9)</f>
         <v>29</v>
       </c>
-      <c r="C38" s="69" t="s">
-        <v>158</v>
-      </c>
-      <c r="D38" s="70" t="s">
-        <v>203</v>
-      </c>
-      <c r="E38" s="70" t="s">
-        <v>58</v>
-      </c>
-      <c r="F38" s="71" t="s">
-        <v>78</v>
-      </c>
-      <c r="G38" s="70" t="s">
-        <v>104</v>
-      </c>
-      <c r="H38" s="71" t="s">
-        <v>123</v>
-      </c>
-      <c r="I38" s="70" t="s">
-        <v>161</v>
-      </c>
-      <c r="J38" s="71" t="s">
-        <v>161</v>
-      </c>
-      <c r="K38" s="70" t="s">
-        <v>161</v>
-      </c>
-      <c r="L38" s="73">
+      <c r="C38" s="68" t="s">
+        <v>155</v>
+      </c>
+      <c r="D38" s="69" t="s">
+        <v>198</v>
+      </c>
+      <c r="E38" s="69" t="s">
+        <v>57</v>
+      </c>
+      <c r="F38" s="70" t="s">
+        <v>77</v>
+      </c>
+      <c r="G38" s="69" t="s">
+        <v>102</v>
+      </c>
+      <c r="H38" s="70" t="s">
+        <v>120</v>
+      </c>
+      <c r="I38" s="69" t="s">
+        <v>158</v>
+      </c>
+      <c r="J38" s="70" t="s">
+        <v>158</v>
+      </c>
+      <c r="K38" s="69" t="s">
+        <v>158</v>
+      </c>
+      <c r="L38" s="72">
         <v>1</v>
       </c>
-      <c r="M38" s="70">
+      <c r="M38" s="69">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N38" s="71">
+      <c r="N38" s="70">
         <v>22</v>
       </c>
-      <c r="O38" s="63" t="s">
-        <v>198</v>
-      </c>
-      <c r="P38" s="74">
+      <c r="O38" s="62" t="s">
+        <v>193</v>
+      </c>
+      <c r="P38" s="73">
         <v>1.06</v>
       </c>
-      <c r="Q38" s="75">
-        <f t="shared" ref="Q38" si="16">P38*N38</f>
+      <c r="Q38" s="74">
+        <f t="shared" ref="Q38" si="15">P38*N38</f>
         <v>23.32</v>
       </c>
-      <c r="R38" s="70"/>
+      <c r="R38" s="69"/>
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
       <c r="B39" s="47">
-        <f>ROW(B39) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="C39" s="59" t="s">
-        <v>158</v>
+      <c r="C39" s="58" t="s">
+        <v>155</v>
       </c>
       <c r="D39" s="38" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="E39" s="38" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F39" s="39" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G39" s="38" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="H39" s="39" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="I39" s="38" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="J39" s="39" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="K39" s="38" t="s">
-        <v>161</v>
-      </c>
-      <c r="L39" s="64">
+        <v>158</v>
+      </c>
+      <c r="L39" s="63">
         <v>1</v>
       </c>
       <c r="M39" s="38">
@@ -3706,10 +3686,10 @@
       <c r="N39" s="39">
         <v>22</v>
       </c>
-      <c r="O39" s="62" t="s">
-        <v>197</v>
-      </c>
-      <c r="P39" s="49">
+      <c r="O39" s="61" t="s">
+        <v>192</v>
+      </c>
+      <c r="P39" s="48">
         <v>0.53300000000000003</v>
       </c>
       <c r="Q39" s="40">
@@ -3718,143 +3698,142 @@
       </c>
       <c r="R39" s="38"/>
     </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
-      <c r="B40" s="48">
-        <f t="shared" si="0"/>
+      <c r="B40" s="64">
+        <f>ROW(B40) - ROW($B$9)</f>
         <v>31</v>
       </c>
-      <c r="C40" s="69" t="s">
-        <v>159</v>
-      </c>
-      <c r="D40" s="70" t="s">
+      <c r="C40" s="68" t="s">
+        <v>156</v>
+      </c>
+      <c r="D40" s="69" t="s">
         <v>31</v>
       </c>
-      <c r="E40" s="70" t="s">
-        <v>60</v>
-      </c>
-      <c r="F40" s="71" t="s">
-        <v>186</v>
-      </c>
-      <c r="G40" s="70" t="s">
-        <v>80</v>
-      </c>
-      <c r="H40" s="71" t="s">
-        <v>124</v>
-      </c>
-      <c r="I40" s="70" t="s">
-        <v>161</v>
-      </c>
-      <c r="J40" s="71" t="s">
-        <v>161</v>
-      </c>
-      <c r="K40" s="70" t="s">
-        <v>139</v>
-      </c>
-      <c r="L40" s="73">
+      <c r="E40" s="69" t="s">
+        <v>59</v>
+      </c>
+      <c r="F40" s="70" t="s">
+        <v>182</v>
+      </c>
+      <c r="G40" s="69" t="s">
+        <v>79</v>
+      </c>
+      <c r="H40" s="70" t="s">
+        <v>121</v>
+      </c>
+      <c r="I40" s="69" t="s">
+        <v>158</v>
+      </c>
+      <c r="J40" s="70" t="s">
+        <v>158</v>
+      </c>
+      <c r="K40" s="69" t="s">
+        <v>136</v>
+      </c>
+      <c r="L40" s="72">
         <v>1</v>
       </c>
-      <c r="M40" s="70">
+      <c r="M40" s="69">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N40" s="71">
+      <c r="N40" s="70">
         <v>22</v>
       </c>
-      <c r="O40" s="63" t="s">
-        <v>199</v>
-      </c>
-      <c r="P40" s="74">
+      <c r="O40" s="62" t="s">
+        <v>194</v>
+      </c>
+      <c r="P40" s="73">
         <v>0.505</v>
       </c>
-      <c r="Q40" s="75">
-        <f t="shared" ref="Q40" si="17">P40*N40</f>
+      <c r="Q40" s="74">
+        <f t="shared" ref="Q40" si="16">P40*N40</f>
         <v>11.11</v>
       </c>
-      <c r="R40" s="70"/>
+      <c r="R40" s="69"/>
     </row>
     <row r="41" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
-      <c r="B41" s="65">
+      <c r="B41" s="64">
         <f>ROW(B41) - ROW($B$9)</f>
         <v>32</v>
       </c>
-      <c r="C41" s="66" t="s">
+      <c r="C41" s="65" t="s">
+        <v>156</v>
+      </c>
+      <c r="D41" s="57" t="s">
+        <v>32</v>
+      </c>
+      <c r="E41" s="57" t="s">
+        <v>60</v>
+      </c>
+      <c r="F41" s="66" t="s">
+        <v>182</v>
+      </c>
+      <c r="G41" s="57" t="s">
+        <v>80</v>
+      </c>
+      <c r="H41" s="66" t="s">
+        <v>122</v>
+      </c>
+      <c r="I41" s="57" t="s">
+        <v>158</v>
+      </c>
+      <c r="J41" s="66" t="s">
+        <v>158</v>
+      </c>
+      <c r="K41" s="57" t="s">
         <v>159</v>
       </c>
-      <c r="D41" s="58" t="s">
-        <v>32</v>
-      </c>
-      <c r="E41" s="58" t="s">
-        <v>61</v>
-      </c>
-      <c r="F41" s="67" t="s">
-        <v>186</v>
-      </c>
-      <c r="G41" s="58" t="s">
-        <v>81</v>
-      </c>
-      <c r="H41" s="67" t="s">
-        <v>125</v>
-      </c>
-      <c r="I41" s="58" t="s">
-        <v>161</v>
-      </c>
-      <c r="J41" s="67" t="s">
-        <v>161</v>
-      </c>
-      <c r="K41" s="58" t="s">
-        <v>162</v>
-      </c>
-      <c r="L41" s="68">
+      <c r="L41" s="67">
         <v>1</v>
       </c>
-      <c r="M41" s="58">
+      <c r="M41" s="57">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
       <c r="N41" s="39">
         <v>22</v>
       </c>
-      <c r="O41" s="62" t="s">
-        <v>198</v>
-      </c>
-      <c r="P41" s="49">
+      <c r="O41" s="61" t="s">
+        <v>193</v>
+      </c>
+      <c r="P41" s="48">
         <v>0.69</v>
       </c>
       <c r="Q41" s="40">
         <f>P41*N41</f>
         <v>15.18</v>
       </c>
-      <c r="R41" s="58"/>
+      <c r="R41" s="57"/>
     </row>
     <row r="42" spans="1:18" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
-      <c r="B42" s="41"/>
-      <c r="C42" s="42"/>
-      <c r="D42" s="43"/>
-      <c r="E42" s="44"/>
-      <c r="F42" s="45"/>
-      <c r="G42" s="46"/>
-      <c r="H42" s="45"/>
-      <c r="I42" s="46"/>
-      <c r="J42" s="45"/>
-      <c r="K42" s="46"/>
-      <c r="L42" s="46"/>
-      <c r="M42" s="46"/>
-      <c r="N42" s="83" t="s">
+      <c r="B42" s="25"/>
+      <c r="C42" s="41"/>
+      <c r="D42" s="42"/>
+      <c r="E42" s="43"/>
+      <c r="F42" s="44"/>
+      <c r="G42" s="45"/>
+      <c r="H42" s="44"/>
+      <c r="I42" s="45"/>
+      <c r="J42" s="44"/>
+      <c r="K42" s="45"/>
+      <c r="L42" s="45"/>
+      <c r="M42" s="45"/>
+      <c r="N42" s="88" t="s">
         <v>5</v>
       </c>
-      <c r="O42" s="84"/>
-      <c r="P42" s="84"/>
-      <c r="Q42" s="50">
+      <c r="O42" s="89"/>
+      <c r="P42" s="89"/>
+      <c r="Q42" s="49">
         <f>SUM(Q10:Q41)</f>
-        <v>536.86219999999992</v>
-      </c>
-      <c r="R42" s="81"/>
+        <v>916.99600000000009</v>
+      </c>
+      <c r="R42" s="86"/>
     </row>
     <row r="43" spans="1:18" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="1"/>
       <c r="B43" s="25"/>
       <c r="C43" s="37"/>
       <c r="D43" s="9"/>
@@ -3867,16 +3846,16 @@
       <c r="K43" s="10"/>
       <c r="L43" s="10"/>
       <c r="M43" s="10"/>
-      <c r="N43" s="83" t="s">
+      <c r="N43" s="88" t="s">
         <v>6</v>
       </c>
-      <c r="O43" s="84"/>
-      <c r="P43" s="84"/>
-      <c r="Q43" s="51">
+      <c r="O43" s="89"/>
+      <c r="P43" s="89"/>
+      <c r="Q43" s="50">
         <f>Q42/20</f>
-        <v>26.843109999999996</v>
-      </c>
-      <c r="R43" s="82"/>
+        <v>45.849800000000002</v>
+      </c>
+      <c r="R43" s="87"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -3909,15 +3888,15 @@
     <hyperlink ref="O32" r:id="rId20"/>
     <hyperlink ref="O33" r:id="rId21"/>
     <hyperlink ref="O34" r:id="rId22"/>
-    <hyperlink ref="O35" r:id="rId23"/>
-    <hyperlink ref="O36" r:id="rId24"/>
-    <hyperlink ref="O37" r:id="rId25"/>
-    <hyperlink ref="O39" r:id="rId26"/>
-    <hyperlink ref="O41" r:id="rId27"/>
-    <hyperlink ref="O38" r:id="rId28"/>
-    <hyperlink ref="O40" r:id="rId29"/>
-    <hyperlink ref="O16" r:id="rId30"/>
-    <hyperlink ref="O31" r:id="rId31"/>
+    <hyperlink ref="O36" r:id="rId23"/>
+    <hyperlink ref="O37" r:id="rId24"/>
+    <hyperlink ref="O39" r:id="rId25"/>
+    <hyperlink ref="O41" r:id="rId26"/>
+    <hyperlink ref="O38" r:id="rId27"/>
+    <hyperlink ref="O40" r:id="rId28"/>
+    <hyperlink ref="O16" r:id="rId29"/>
+    <hyperlink ref="O31" r:id="rId30"/>
+    <hyperlink ref="O35" r:id="rId31"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId32"/>

</xml_diff>